<commit_message>
feat: role-based limits, printable Rx pad, active/inactive status, doctor patient deletion, and mobile UI responsiveness
</commit_message>
<xml_diff>
--- a/public/OBGYN_Clinic_Database.xlsx
+++ b/public/OBGYN_Clinic_Database.xlsx
@@ -512,7 +512,7 @@
         <v>Nov 17, 2026</v>
       </c>
       <c r="M2" t="str">
-        <v>28w 6d</v>
+        <v>29w 0d</v>
       </c>
       <c r="N2" t="str">
         <v>3rd</v>
@@ -565,7 +565,7 @@
         <v>Jan 10, 2027</v>
       </c>
       <c r="M3" t="str">
-        <v>21w 1d</v>
+        <v>21w 2d</v>
       </c>
       <c r="N3" t="str">
         <v>2nd</v>
@@ -577,7 +577,7 @@
         <v>Primigravida. Pre-existing Subclinical Hypothyroidism managed with Levothyroxine 50mcg daily.</v>
       </c>
       <c r="Q3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -618,7 +618,7 @@
         <v>Mar 27, 2027</v>
       </c>
       <c r="M4" t="str">
-        <v>10w 2d</v>
+        <v>10w 3d</v>
       </c>
       <c r="N4" t="str">
         <v>1st</v>
@@ -642,7 +642,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -856,31 +856,31 @@
         <v>Elena Reyes-Dizon</v>
       </c>
       <c r="C6" t="str">
-        <v>chk-1788156339667</v>
+        <v>chk-1788256920901</v>
       </c>
       <c r="D6" t="str">
-        <v>2026-08-31</v>
+        <v>2026-09-01</v>
       </c>
       <c r="E6" t="str">
-        <v>23</v>
-      </c>
-      <c r="F6">
-        <v>23</v>
-      </c>
-      <c r="G6">
-        <v>23</v>
+        <v>N/A</v>
+      </c>
+      <c r="F6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G6" t="str">
+        <v>N/A</v>
       </c>
       <c r="H6" t="str">
         <v>N/A</v>
       </c>
       <c r="I6" t="str">
-        <v>sdsdsd</v>
+        <v>Triage Vitals Check (Clinical Assistant)</v>
       </c>
       <c r="J6" t="str">
-        <v>sdsdsd</v>
+        <v>Vital Signs &amp; Prep</v>
       </c>
       <c r="K6" t="str">
-        <v>2026-11-30</v>
+        <v>As needed</v>
       </c>
       <c r="L6" t="str">
         <v/>
@@ -894,39 +894,77 @@
         <v>Elena Reyes-Dizon</v>
       </c>
       <c r="C7" t="str">
-        <v>chk-102-2</v>
+        <v>chk-1788156339667</v>
       </c>
       <c r="D7" t="str">
-        <v>2026-08-10</v>
+        <v>2026-08-31</v>
       </c>
       <c r="E7" t="str">
-        <v>112/74</v>
+        <v>23</v>
       </c>
       <c r="F7">
-        <v>59.2</v>
+        <v>23</v>
       </c>
       <c r="G7">
-        <v>150</v>
+        <v>23</v>
       </c>
       <c r="H7" t="str">
         <v>N/A</v>
       </c>
       <c r="I7" t="str">
-        <v>18 Weeks Gestation, Normal Anatomy Scan</v>
+        <v>sdsdsd</v>
       </c>
       <c r="J7" t="str">
-        <v>Congenital Anomaly Scan (Level II Ultrasound)</v>
+        <v>sdsdsd</v>
       </c>
       <c r="K7" t="str">
-        <v>2026-09-08</v>
+        <v>2026-11-30</v>
       </c>
       <c r="L7" t="str">
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>pat-102</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Elena Reyes-Dizon</v>
+      </c>
+      <c r="C8" t="str">
+        <v>chk-102-2</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2026-08-10</v>
+      </c>
+      <c r="E8" t="str">
+        <v>112/74</v>
+      </c>
+      <c r="F8">
+        <v>59.2</v>
+      </c>
+      <c r="G8">
+        <v>150</v>
+      </c>
+      <c r="H8" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I8" t="str">
+        <v>18 Weeks Gestation, Normal Anatomy Scan</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Congenital Anomaly Scan (Level II Ultrasound)</v>
+      </c>
+      <c r="K8" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>